<commit_message>
feat: preencher dados dinamicos no anexo do memorial fotografico
</commit_message>
<xml_diff>
--- a/src/planilha_monitoramento.xlsx
+++ b/src/planilha_monitoramento.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-20580" yWindow="1365" windowWidth="13740" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoramento" sheetId="1" state="visible" r:id="rId1"/>
@@ -581,7 +581,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>08/06/2025</t>
+          <t>06/08/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09/06/2025</t>
+          <t>06/09/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10/06/2025</t>
+          <t>06/10/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11/03/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12/06/2026</t>
+          <t>06/12/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>12/06/2027</t>
+          <t>06/12/2027</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>12/06/2027</t>
+          <t>06/12/2027</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">

</xml_diff>

<commit_message>
feat: altera fonte de dados para utilizar segunda planilha
</commit_message>
<xml_diff>
--- a/src/planilha_monitoramento.xlsx
+++ b/src/planilha_monitoramento.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monitoramento" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,24 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -54,27 +43,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -102,33 +76,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -496,15 +449,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="37" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="37" customWidth="1" min="7" max="7"/>
     <col width="37" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -514,62 +467,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Cidade</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Pessoal Responsável</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Matriculas das Pessoas Responsáveis</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Coordenador</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Contrato</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Assinatura</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Relatório Gerado</t>
         </is>
@@ -581,17 +534,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06/08/2025</t>
+          <t>12/06/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10:00:06</t>
+          <t>10:00:19</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Joao Recife Pessoas</t>
+          <t>Recife</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -601,7 +554,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
+          <t>Alcides Vieira e Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0000001/00;000002/00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -611,762 +569,20 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Nº 1.041.080/14</t>
+          <t>Nº 1.041.080/10</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>26/04/2025 a 01/05/2031</t>
+          <t>26/04/2025 a 01/05/2043</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
+          <t>Débora Marcolino;Enildo Manoel</t>
         </is>
       </c>
       <c r="L2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06/09/2025</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>10:00:07</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/15</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2032</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>06/10/2025</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>10:00:08</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/16</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2033</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>03/11/2025</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>10:50:00</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Recife</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/08</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>22/09/2025 a 26/09/2025</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>06/12/2025</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>10:00:10</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/18</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2035</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>06/12/2025</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>10:00:11</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/19</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2036</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>06/12/2025</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>10:00:12</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/20</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2037</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>06/12/2025</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>10:00:13</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/21</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2038</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>06/12/2025</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>10:00:14</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/22</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2039</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>06/12/2025</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>10:00:15</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Joao Recife Pessoas</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/23</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2040</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>06/12/2025</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>10:00:16</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Recife</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Alcides Vieira, Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/24</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2041</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Alcides Vieira;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>06/12/2025</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>10:00:17</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Recife</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Débora Marcolino e Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/08</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2041</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Débora Marcolino;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>06/12/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>10:00:18</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Recife</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Débora Marcolino e Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/09</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2042</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Débora Marcolino;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>15</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>06/12/2027</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>10:00:19</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Recife</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Débora Marcolino e Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/10</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2043</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Débora Marcolino;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>17</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>06/12/2027</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>10:00:19</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Recife</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Terminal Rodoviário do Recife - TIP</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Alcides Vieira e Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>0000001/00;000002/00</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Maria Ângela Albuquerque de Freitas</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Nº 1.041.080/10</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>26/04/2025 a 01/05/2043</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Débora Marcolino;Enildo Manoel</t>
-        </is>
-      </c>
-      <c r="L16" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1385,16 +601,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" style="4" min="2" max="2"/>
-    <col width="26" customWidth="1" style="5" min="3" max="3"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" style="5" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
@@ -1414,27 +630,23 @@
           <t>Processo SEI Nº</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Carta SAP/PER/ARPE Nº</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Doc. SEI Nº</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Periodo de Vistoria da ARPE</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="n">
         <v>2</v>
@@ -1499,27 +711,32 @@
       <c r="A15" t="n">
         <v>15</v>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>01/2025</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>17</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>01/2025</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>0.000.000/00</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>0000000000.0000000000/00</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>001/2025;002/2025</t>
         </is>
@@ -1527,15 +744,14 @@
       <c r="F16" t="n">
         <v>12345678</v>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>01 A 22/09/2025;  30/09/2025</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1545,274 +761,182 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K95"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="61" customWidth="1" min="3" max="3"/>
-    <col width="526" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="533" customWidth="1" min="11" max="11"/>
+    <col width="296" customWidth="1" min="3" max="3"/>
+    <col width="312" customWidth="1" min="4" max="4"/>
+    <col width="241" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="498" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>ID da não conformidade</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Não Conformidade</t>
-        </is>
-      </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Informação SOCICAM</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Constatação</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Análise da Arpe</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Informação SOCICAM carta</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Vistoria da Arpe</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Situação</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>Terminal de Petrolina</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>1</v>
-      </c>
       <c r="B6" t="inlineStr">
         <is>
           <t>Terminal de Caruaru</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>1</v>
-      </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>1</v>
-      </c>
       <c r="B9" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>1</v>
-      </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>1</v>
-      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1827,12 +951,7 @@
           <t>Terminal de Caruaru</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1847,12 +966,7 @@
           <t>Terminal de Garanhuns</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1867,12 +981,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1887,12 +996,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1907,12 +1011,7 @@
           <t>Terminal de Garanhuns</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1927,12 +1026,7 @@
           <t>Terminal de Garanhuns</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1947,12 +1041,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1967,12 +1056,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -1987,12 +1071,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2007,12 +1086,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2027,12 +1101,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2047,12 +1116,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2067,12 +1131,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2087,12 +1146,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2107,12 +1161,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2127,12 +1176,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2147,12 +1191,7 @@
           <t>Terminal de Arcoverde</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
@@ -2167,12 +1206,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Infiltração na coluna de sustentação da estrutura metálica da área de embarque e desembarque do Terminal do Recife (TIP), conforme evidenciado nas fotos 01 e 02, a seguir!!!!!!!</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Infiltração em coluna de sustentação do Terminal do Recife em 20/03/2025.;Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2187,11 +1221,6 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Falta de manutenção adequada no banheiro feminino para PCD localizado no primeiro andar do Terminal do Recife (TIP), conforme detalhado.</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2202,11 +1231,6 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Espelho oxidado, conforme evidenciado na foto 03, a seguir. </t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2217,11 +1241,6 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Barra oxidada em torno da pian cofnorme foto 01 e foto 02. </t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2232,12 +1251,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Barra de apoio vertical oxidada, conforme foto 04, a seguir. </t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>Espelho e barra em torno da pia oxidados no banehiro feminino PCD do Terminal de Recife, 20/03/2025;Infiltração em coluna de sustentação do Terminal do Recife em 20/03/2025</t>
         </is>
@@ -2252,12 +1266,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2272,12 +1281,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2292,12 +1296,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2312,12 +1311,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2332,12 +1326,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2352,12 +1341,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2372,12 +1356,7 @@
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2392,12 +1371,7 @@
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2412,12 +1386,7 @@
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2432,12 +1401,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2452,12 +1416,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2472,12 +1431,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2492,12 +1446,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2512,12 +1461,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2532,12 +1476,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2552,12 +1491,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2572,12 +1506,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2592,12 +1521,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2612,12 +1536,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2632,12 +1551,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2652,12 +1566,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2672,12 +1581,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2692,12 +1596,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2712,12 +1611,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. ;Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. ;Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2732,12 +1626,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2752,12 +1641,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2772,11 +1656,6 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2787,12 +1666,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>Piso desgastado conforme evidência da foto 04.</t>
         </is>
@@ -2807,11 +1681,6 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2822,12 +1691,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
+      <c r="I63" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2842,12 +1706,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
+      <c r="I64" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2862,12 +1721,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
+      <c r="I65" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2882,12 +1736,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
+      <c r="I66" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2902,12 +1751,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
+      <c r="I67" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2922,12 +1766,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
+      <c r="I68" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2942,12 +1781,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
+      <c r="I69" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2962,12 +1796,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
+      <c r="I70" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -2982,12 +1811,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
+      <c r="I71" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3002,12 +1826,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
+      <c r="I72" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3022,12 +1841,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
+      <c r="I73" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3042,12 +1856,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3062,12 +1871,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
+      <c r="I75" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3082,12 +1886,7 @@
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
+      <c r="I76" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3102,12 +1901,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
+      <c r="I77" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3122,12 +1916,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
+      <c r="I78" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3142,12 +1931,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
+      <c r="I79" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3162,12 +1946,7 @@
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K80" t="inlineStr">
+      <c r="I80" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3182,12 +1961,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
+      <c r="I81" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3202,12 +1976,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
+      <c r="I82" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3222,12 +1991,7 @@
           <t>Terminal de Arcoverde (ARC)</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
+      <c r="I83" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3242,12 +2006,7 @@
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K84" t="inlineStr">
+      <c r="I84" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3262,12 +2021,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
+      <c r="I85" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3282,12 +2036,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
+      <c r="I86" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3302,12 +2051,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
+      <c r="I87" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3322,12 +2066,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr">
+      <c r="I88" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3342,12 +2081,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K89" t="inlineStr">
+      <c r="I89" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3362,12 +2096,7 @@
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr">
+      <c r="I90" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3382,12 +2111,7 @@
           <t>Terminal de Serra Talhada (SER)</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr">
+      <c r="I91" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
         </is>
@@ -3395,7 +2119,7 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -3404,52 +2128,57 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>TIP_2025_01;TIP_2025_02;TIP_2025_03;TIP_2025_04;TIP_2025_05</t>
+          <t>A SOCICAM informou que o serviço estava em andamento com a equipe interna de manutenção, com previsão de conclusão em setembro de 2025 (Carta SAP/PER/ARPE N° 002/2025).; A SOCICAM informou que os serviços estavam em andamento com prazo previsto para julho/2025 (Carta SAP/PER/ARPE N° 002/2025).</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Base do suporte da sinalização em braile enferrujada e desatualizada na área de embarque e desembarque do Terminal de Recife (TIP), conforme evidenciado nas Fotos 01 e 02, a seguir.; Falta de manutenção adequada no banheiro masculino para PCD localizado no térreo do Terminal de Recife (TIP), conforme detalhado.;Saboneteira ausente, a seguir na Fotos 03 e 04.; Pia com vazamento, conforme a Fotos 03 e 04.;Fachada interna necessitando de pintura do Terminal de Recife (TIP), conforme evidenciado na Fotos 05 e 06, a seguir.</t>
+          <t>O serviço de pintura está em andamento, conforme demonstrado no Memorial Fotográfico pelo comparativo entre a Foto 01 de 18/06/2025 e a Foto 02 de 30/09/2025.; A pintura na porta foi finalizada, conforme demonstra o Memorial Fotográfico pelo comparativo entre a Foto 05 de 18/06/2025 e a Foto 06 de 30/09/2025.</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Não Conformidade pendente. Recomenda-se que a SOCICAM encaminhe comprovação de conclusão desses serviços, que se encontram em atraso considerando a informação da SOCICAM constante da Carta SAP/PER/ARPE N° 002/2025.;Não Conformidade sanada.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM; lalala;hahaha;pipipip</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>LOREM IPSUM;LOREM IPSUM; lalala;hahaha;pipipip</t>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>Suporte da sinalização em braile enferrujada do Terminal do Recife em 30/09/2025:sinalização em braile enferrujada do Terminal do Recife em 30/09/2025;Pia com vazamento e saboneteira quebrada no banheiro do térreo masculino para PCD do Terminal de Recife em 30/09/2025:vazamento e saboneteira quebrada no banheiro do térreo masculino para PCD do Terminal de Recife ;Pintura da fachada  do pátio interno desgastada no Terminal de Recife em 30/09/202510/11/2025:fachada do pátio interno desgastada no Terminal de Recife em 30/09/2025</t>
+          <t>Infiltração em coluna de sustentação da estrutura metálica da área de embarque e desembarque; Falta de manutenção adequada no banheiro feminino para PCD localizado no primeiro andar do Terminal de Recife (TIP);  Porta com avaria no banheiro feminino do primeiro andar do Terminal de Recife (TIP).;Pintura do meio-fio desgastada na área de circulação e manobra dos ônibus; Falta de manutenção adequada na infraestrutura do ponto de embarque e desembarque.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
           <t>Terminal de Caruaru (CAR)</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>CAR_2025_00;CAR_2025_08;CAR_2025_10</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>Placas do teto do terminal apresentando descolamentos no pátio de manobras do Terminal de Caruaru, conforme evidenciado na Foto 07 e foto 08, a seguir.; Viga apresentando rachaduras próximo a juntas da testeira necessitando de reparo estrutural no pátio de manobras do Terminal de Caruaru, conforme evidenciado na Fotos 09 e 10, a seguir.</t>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -3459,37 +2188,27 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>Placas descoladas no Terminal de Caruaru em 25/09/2025.;Placas descoladas no Terminal de Caruaru em 25/09/2025.;Rachaduras próximas à junta de dilatação na testeira do pátio de manobras no Terminal de Caruaru em 25/09/2025.;Detalhe das rachaduras na testeira do pátio de manobras no Terminal de Caruaru em 25/09/2025.</t>
+          <t>Área precisando de capinação no pátio de manobras; Área precisando de capinação no terreno lateral do Terminal; Área com infiltração na fachada lateral do Terminal;  Pintura desgastada no muro e na grade do pátio de manobra no Terminal;  Pintura desgastada no muro lateral no Terminal; Vidraças na parte administrativa precisando de limpeza; Meio-fio desgastado na entrada do Terminal;Rampa para PCD desgastada no Terminal;Desgaste do pavimento na rampa de carga e descarga na entrada do Terminal</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
           <t>Terminal de Garanhuns (GAR)</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>GAR_2025_07;GAR_2025_09</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Vigas da testeira necessitando de manutenção estrutural no pátio de manobras do Terminal de Garanhuns, conforme evidenciado nas Fotos 11 e 12.;Viga deteriorada na fachada lateral com armadura de ferro exposta no pátio de manobras do Terminal de Garanhuns, conforme evidenciado nas Fotos 13 e 14.</t>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -3499,37 +2218,28 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>Vigas da testeira necessitando de manutenção estrutural no Terminal de Garanhuns em 22/09/2025;Vigas da testeira necessitando de manutenção estrutural no Terminal de Garanhuns em 22/09/2025.;Viga com armadura de ferro exposta no Terminal de Garanhuns em 22/09/2025;Viga com armadura de ferro exposta no Terminal de Garanhuns em 22/09/2025.</t>
+          <t xml:space="preserve">Pintura desgastada no muro da lateral do Terminal; Pintura desgastada do muro do pátio de manobras no Terminal;Pintura desgastada das colunas da entrada do Terminal; Pintura desgastada nas colunas da fachada do lado do pátio de manobras no Terminal;Pintura desgastada na parede lateral direita no Terminal
+</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
           <t>Terminal de Petrolina (PET)</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>PET_2025_01;PET_2025_06</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>Fachada necessitando de manutenção e limpeza na entrada do Terminal de Petrolina, conforme evidenciado nas Fotos 15 e 16.;Falta de Limpeza dos vidros do Terminal de Petrolina, conforme evidenciado nas Fotos 17 e 18.</t>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -3537,19 +2247,46 @@
           <t>LOREM IPSUM;LOREM IPSUM</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr">
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>1</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Terminal de Arcoverde (ARC)</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
         <is>
           <t>LOREM IPSUM</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr">
+      <c r="H96" t="inlineStr">
         <is>
           <t>LOREM IPSUM;LOREM IPSUM</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>Fachada necessitando de manutenção e limpeza no Terminal de Petrolina em 24/09/2025.;Fachada necessitando de manutenção e limpeza no Terminal de Petrolina em 24/09/2025.;Vidros necessitando de limpeza no Terminal de Petrolina em 24/09/2025.;Vidros necessitando de limpeza no Terminal de Petrolina em 24/09/2025.</t>
+    </row>
+    <row r="97">
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>LOREM IPSUM;LOREM IPSUM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FIX: Corrige IndexError em loop de agregação do resumo.
</commit_message>
<xml_diff>
--- a/src/planilha_monitoramento.xlsx
+++ b/src/planilha_monitoramento.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -582,8 +582,70 @@
           <t>Débora Marcolino;Enildo Manoel</t>
         </is>
       </c>
-      <c r="L2" t="b">
-        <v>1</v>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>VERDADEIRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>09/06/2025</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10:00:07</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário do Recife - TIP</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Alcides Vieira e Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0000002/00;000002/00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Maria Ângela Albuquerque de Freitas</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Nº 1.041.080/10</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>26/04/2025 a 01/05/2043</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Débora Marcolino;Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>VERDADEIRO</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2158,7 +2220,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Infiltração em coluna de sustentação da estrutura metálica da área de embarque e desembarque; Falta de manutenção adequada no banheiro feminino para PCD localizado no primeiro andar do Terminal de Recife (TIP);  Porta com avaria no banheiro feminino do primeiro andar do Terminal de Recife (TIP).;Pintura do meio-fio desgastada na área de circulação e manobra dos ônibus; Falta de manutenção adequada na infraestrutura do ponto de embarque e desembarque.</t>
+          <t>Infiltração em coluna de sustentação da estrutura metálica da área de embarque e desembarque: Falta de manutenção adequada no banheiro feminino para PCD localizado no primeiro andar do Terminal de Recife (TIP);  Porta com avaria no banheiro feminino do primeiro andar do Terminal de Recife (TIP).;Pintura do meio-fio desgastada na área de circulação e manobra dos ônibus; Falta de manutenção adequada na infraestrutura do ponto de embarque e desembarque.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: ajustes na visualização das ncs
</commit_message>
<xml_diff>
--- a/src/planilha_monitoramento.xlsx
+++ b/src/planilha_monitoramento.xlsx
@@ -2286,14 +2286,6 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="n">
-        <v>1</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Terminal de Petrolina (PET)</t>
-        </is>
-      </c>
       <c r="F95" t="inlineStr">
         <is>
           <t>LOREM IPSUM;LOREM IPSUM</t>
@@ -2311,14 +2303,6 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="n">
-        <v>1</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Terminal de Arcoverde (ARC)</t>
-        </is>
-      </c>
       <c r="F96" t="inlineStr">
         <is>
           <t>LOREM IPSUM;LOREM IPSUM</t>

</xml_diff>

<commit_message>
fix: resolve problema de NCs não encontradas devido a filtro estrito de terminal
</commit_message>
<xml_diff>
--- a/src/planilha_monitoramento.xlsx
+++ b/src/planilha_monitoramento.xlsx
@@ -76,11 +76,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -470,62 +467,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Cidade</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Pessoal Responsável</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Matriculas das Pessoas Responsáveis</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Coordenador</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Contrato</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Assinatura</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Relatório Gerado</t>
         </is>
@@ -615,37 +612,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Processo CTR Nº</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Contrato de Concessão Nº</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Processo SEI Nº</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Carta SAP/PER/ARPE Nº</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Doc. SEI Nº</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Periodo de Vistoria da ARPE</t>
         </is>
@@ -695,7 +692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -706,51 +703,51 @@
     <col width="48" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="498" customWidth="1" min="9" max="9"/>
+    <col width="1534" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Informação SOCICAM</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Constatação</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Análise da Arpe</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Informação SOCICAM carta</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Vistoria da Arpe</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Situação</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>
@@ -797,7 +794,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Infiltração em coluna de sustentação da estrutura metálica da área de embarque e desembarque: Falta de manutenção adequada no banheiro feminino para PCD localizado no primeiro andar do Terminal de Recife (TIP);  Porta com avaria no banheiro feminino do primeiro andar do Terminal de Recife (TIP).;Pintura do meio-fio desgastada na área de circulação e manobra dos ônibus; Falta de manutenção adequada na infraestrutura do ponto de embarque e desembarque.</t>
+          <t>Situação da infiltração em coluna de sustentação do Terminal de Recife em 18/06/2025.:Situação da coluna de sustentação em processo de restauração no Terminal de Recife em 30/09/2025.;Barras repintadas, mas espelho ainda oxidado no banheiro feminino para PCD do Terminal de Recife em 18/06/2025: Espelho substituído no banheiro feminino para PCD 30/09/2025.;Porta com avaria no banheiro feminino no Terminal de Recife em 18/06/2025.:Porta restaurada no banheiro feminino no Terminal de Recife em 30/09/2025.;Detalhe da pintura do meio-fio iniciada no pátio interno no Terminal de Recife 18/06/2025.: Detalhe da pintura do meio-fio em andamento no pátio interno no Terminal de Recife 30/09/2025.;Pintura da faixa de pedestres iniciada, na entrada do Terminal de Recife em 18/06/2025.:Pintura da faixa de pedestres finalizada, na entrada do Terminal de Recife em 30/09/2025.: Parada de ônibus com pintura desgastada na entrada do Terminal de Recife em 18/06/2025.:Parada de ônibus com pintura desgastada na entrada do Terminal de Recife em 30/09/2025.</t>
         </is>
       </c>
     </row>
@@ -827,7 +824,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Área precisando de capinação no pátio de manobras; Área precisando de capinação no terreno lateral do Terminal; Área com infiltração na fachada lateral do Terminal;  Pintura desgastada no muro e na grade do pátio de manobra no Terminal;  Pintura desgastada no muro lateral no Terminal; Vidraças na parte administrativa precisando de limpeza; Meio-fio desgastado na entrada do Terminal;Rampa para PCD desgastada no Terminal;Desgaste do pavimento na rampa de carga e descarga na entrada do Terminal</t>
+          <t xml:space="preserve"> Falta de capinação no pátio de manobras do Terminal de Caruaru em 09/06/2025.:Capinação feita no pátio de manobras do Terminal de Caruaru em 25/09/2025.;Falta capinação no terreno lateral do Terminal de Caruaru em 09/06/2025.:Capinação feita no terreno lateral do Terminal de Caruaru em 25/09/2025.;Detalhe da infiltração na parte lateral do Terminal de Caruaru em 09/06/2025.:Infiltração continua na parte lateral do Terminal de Caruaru em 25/09/2025.;Muro e grade internos com pinturas desgastadas no pátio de manobras do Terminal de Caruaru em 09/06/2025.:Muro e grade internos continuam com pinturas desgastadas no pátio de manobras do Terminal de Caruaru em 25/09/2025.; Muro e grade internos com pinturas desgastadas no pátio de manobras do Terminal de Caruaru em 09/06/2025..:Muro externo continua com pintura desgastada no Terminal de Caruaru em 25/09/2025.;Vidraças na parte administrativa precisando de limpeza no Terminal de Caruaru em 09/06/2025.:Vidraças na parte administrativa limpas no Terminal de Caruaru em 25/09/2025.;Meio-fio desgastado na entrada do Terminal de Caruaru em 09/06/2025.:Meio-fio continua desgastado na entrada do Terminal de Caruaru em 25/09/2025.;Rampa para PCD desgastada no Terminal de Caruaru em 09/06/2025.:Rampa para PCD continua desgastada no Terminal de Caruaru em 25/09/2025.;Rampa de carga e descarga com desgaste no pavimento na entrada do Terminal de Caruaru em 09/06/2025.:Rampa de carga e descarga continua com desgaste no pavimento na entrada do Terminal de Caruaru em 25/09/2025.</t>
         </is>
       </c>
     </row>
@@ -857,59 +854,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>"Pintura desgastada no muro da lateral do Terminal; Pintura desgastada do muro do pátio de manobras no Terminal;Pintura desgastada das colunas da entrada do Terminal; Pintura desgastada nas colunas da fachada do lado do pátio de manobras no Terminal;Pintura desgastada na parede lateral direita no Terminal
-"</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>LOREM IPSUM;LOREM IPSUM</t>
+          <t>Pintura desgastada do muro da lateral no Terminal de Garanhuns em 12/06/2025.:Pintura continua desgastada do muro da lateral no Terminal de Garanhuns em 22/09/2025;Pintura desgastada do muro da entrada do pátio de manobras no Terminal de Garanhuns em 12/06/2025.:Pintura continua desgastada do muro da entrada do pátio de manobras no Terminal de Garanhuns em 22/09/2025.;Pintura desgastada das colunas da entrada do Terminal de Garanhuns em 12/06/2025.:Pintura realizada das colunas da entrada do Terminal de Garanhuns em 22/09/2025.;Pintura desgastada nas colunas do pátio de manobras do Terminal de Garanhuns em 12/06/2025.:Pintura realizada nas colunas do pátio de manobras do Terminal de Garanhuns em 22/09/2025.; Pintura desgastada na parede lateral direita do Terminal de Garanhuns em 12/06/2025.:Pintura continua desgastada na parede lateral direita do Terminal de Garanhuns em 22/09/2025</t>
         </is>
       </c>
     </row>

</xml_diff>